<commit_message>
Update Mazandasht work panel and financial workbooks
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Mazandasht_Tamplate V00/INFO.xlsx
+++ b/Mazandasht_Tamplate V00/INFO.xlsx
@@ -6594,7 +6594,7 @@
         <v>1471</v>
       </c>
       <c r="C7" s="14">
-        <v>0</v>
+        <v>6018890069</v>
       </c>
       <c r="D7" s="14" t="s">
         <v>989</v>
@@ -6643,7 +6643,7 @@
         <v>1473</v>
       </c>
       <c r="C10" s="15">
-        <v>0</v>
+        <v>1029303</v>
       </c>
       <c r="D10" s="15" t="s">
         <v>989</v>
@@ -6673,7 +6673,7 @@
         <v>1475</v>
       </c>
       <c r="C12" s="15">
-        <v>0</v>
+        <v>38482872871</v>
       </c>
       <c r="D12" s="15" t="s">
         <v>989</v>
@@ -14207,7 +14207,7 @@
     <tabColor rgb="FF558B2F"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
@@ -14269,6 +14269,11 @@
       <c r="E5" s="3" t="s">
         <v>1324</v>
       </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>وزن تار (کیلوگرم)</t>
+        </is>
+      </c>
     </row>
     <row r="6" spans="1:5" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
@@ -14285,6 +14290,11 @@
       </c>
       <c r="E6" s="4" t="s">
         <v>1327</v>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Tare weight (kg)</t>
+        </is>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
@@ -14300,6 +14310,7 @@
         <f t="shared" ref="E7:E36" si="0">IF($A7="","",$A7&amp;" – "&amp;IF($B7="","(بدون عنوان)",$B7))</f>
         <v>BK01 – 6ک مشکی</v>
       </c>
+      <c r="F7" s="14"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
@@ -14314,6 +14325,7 @@
         <f t="shared" si="0"/>
         <v>BK02 – درب6ک</v>
       </c>
+      <c r="F8" s="15"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
@@ -14328,6 +14340,7 @@
         <f t="shared" si="0"/>
         <v>BK03 – 9ک مشکی</v>
       </c>
+      <c r="F9" s="14"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
@@ -14342,6 +14355,7 @@
         <f t="shared" si="0"/>
         <v>BK04 – ریلی کوچک آبی</v>
       </c>
+      <c r="F10" s="15"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
@@ -14356,6 +14370,7 @@
         <f t="shared" si="0"/>
         <v>BK05 – تک رج آبی بزرگ</v>
       </c>
+      <c r="F11" s="14"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
@@ -14370,6 +14385,7 @@
         <f t="shared" si="0"/>
         <v>BK06 – آبی25*20</v>
       </c>
+      <c r="F12" s="15"/>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" s="5" t="s">
@@ -14384,6 +14400,7 @@
         <f t="shared" si="0"/>
         <v>BK07 – 8ک مشکی</v>
       </c>
+      <c r="F13" s="14"/>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" s="5" t="s">
@@ -14396,6 +14413,7 @@
         <f t="shared" si="0"/>
         <v>BK08 – (بدون عنوان)</v>
       </c>
+      <c r="F14" s="15"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" s="5" t="s">
@@ -14408,6 +14426,7 @@
         <f t="shared" si="0"/>
         <v>BK09 – (بدون عنوان)</v>
       </c>
+      <c r="F15" s="14"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" s="5" t="s">
@@ -14420,6 +14439,7 @@
         <f t="shared" si="0"/>
         <v>BK10 – (بدون عنوان)</v>
       </c>
+      <c r="F16" s="15"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" s="5" t="s">
@@ -14432,6 +14452,7 @@
         <f t="shared" si="0"/>
         <v>BK11 – (بدون عنوان)</v>
       </c>
+      <c r="F17" s="14"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" s="5" t="s">
@@ -14444,6 +14465,7 @@
         <f t="shared" si="0"/>
         <v>BK12 – (بدون عنوان)</v>
       </c>
+      <c r="F18" s="15"/>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" s="5" t="s">
@@ -14456,6 +14478,7 @@
         <f t="shared" si="0"/>
         <v>BK13 – (بدون عنوان)</v>
       </c>
+      <c r="F19" s="14"/>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" s="5" t="s">
@@ -14468,6 +14491,7 @@
         <f t="shared" si="0"/>
         <v>BK14 – (بدون عنوان)</v>
       </c>
+      <c r="F20" s="15"/>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A21" s="5" t="s">
@@ -14480,6 +14504,7 @@
         <f t="shared" si="0"/>
         <v>BK15 – (بدون عنوان)</v>
       </c>
+      <c r="F21" s="14"/>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A22" s="5" t="s">
@@ -14492,6 +14517,7 @@
         <f t="shared" si="0"/>
         <v>BK16 – (بدون عنوان)</v>
       </c>
+      <c r="F22" s="15"/>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A23" s="5" t="s">
@@ -14504,6 +14530,7 @@
         <f t="shared" si="0"/>
         <v>BK17 – (بدون عنوان)</v>
       </c>
+      <c r="F23" s="14"/>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A24" s="5" t="s">
@@ -14516,6 +14543,7 @@
         <f t="shared" si="0"/>
         <v>BK18 – (بدون عنوان)</v>
       </c>
+      <c r="F24" s="15"/>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25" s="5" t="s">
@@ -14528,6 +14556,7 @@
         <f t="shared" si="0"/>
         <v>BK19 – (بدون عنوان)</v>
       </c>
+      <c r="F25" s="14"/>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A26" s="5" t="s">
@@ -14540,6 +14569,7 @@
         <f t="shared" si="0"/>
         <v>BK20 – (بدون عنوان)</v>
       </c>
+      <c r="F26" s="15"/>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A27" s="5" t="s">
@@ -14552,6 +14582,7 @@
         <f t="shared" si="0"/>
         <v>BK21 – (بدون عنوان)</v>
       </c>
+      <c r="F27" s="14"/>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A28" s="5" t="s">
@@ -14564,6 +14595,7 @@
         <f t="shared" si="0"/>
         <v>BK22 – (بدون عنوان)</v>
       </c>
+      <c r="F28" s="15"/>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A29" s="5" t="s">
@@ -14576,6 +14608,7 @@
         <f t="shared" si="0"/>
         <v>BK23 – (بدون عنوان)</v>
       </c>
+      <c r="F29" s="14"/>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A30" s="5" t="s">
@@ -14588,6 +14621,7 @@
         <f t="shared" si="0"/>
         <v>BK24 – (بدون عنوان)</v>
       </c>
+      <c r="F30" s="15"/>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A31" s="5" t="s">
@@ -14600,6 +14634,7 @@
         <f t="shared" si="0"/>
         <v>BK25 – (بدون عنوان)</v>
       </c>
+      <c r="F31" s="14"/>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A32" s="5" t="s">
@@ -14612,6 +14647,7 @@
         <f t="shared" si="0"/>
         <v>BK26 – (بدون عنوان)</v>
       </c>
+      <c r="F32" s="15"/>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A33" s="5" t="s">
@@ -14624,6 +14660,7 @@
         <f t="shared" si="0"/>
         <v>BK27 – (بدون عنوان)</v>
       </c>
+      <c r="F33" s="14"/>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A34" s="5" t="s">
@@ -14636,6 +14673,7 @@
         <f t="shared" si="0"/>
         <v>BK28 – (بدون عنوان)</v>
       </c>
+      <c r="F34" s="15"/>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A35" s="5" t="s">
@@ -14648,6 +14686,7 @@
         <f t="shared" si="0"/>
         <v>BK29 – (بدون عنوان)</v>
       </c>
+      <c r="F35" s="14"/>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A36" s="5" t="s">
@@ -14660,6 +14699,7 @@
         <f t="shared" si="0"/>
         <v>BK30 – (بدون عنوان)</v>
       </c>
+      <c r="F36" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -18322,41 +18362,25 @@
       <c r="F10" s="8"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A11" s="5" t="s">
-        <v>364</v>
-      </c>
+      <c r="A11" s="5"/>
       <c r="B11" s="12" t="str">
         <f>IF($A11="","",IFERROR(IF(VLOOKUP($A11,Accounts!$A$7:$D$566,4,0)="","—",VLOOKUP($A11,Accounts!$A$7:$D$566,4,0)),"—"))</f>
         <v>رضا کاظمی (نمونه)</v>
       </c>
-      <c r="C11" s="6" t="s">
-        <v>315</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>169</v>
-      </c>
-      <c r="E11" s="6" t="s">
-        <v>365</v>
-      </c>
+      <c r="C11" s="6"/>
+      <c r="D11" s="6"/>
+      <c r="E11" s="6"/>
       <c r="F11" s="6"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A12" s="5" t="s">
-        <v>366</v>
-      </c>
+      <c r="A12" s="5"/>
       <c r="B12" s="12" t="str">
         <f>IF($A12="","",IFERROR(IF(VLOOKUP($A12,Accounts!$A$7:$D$566,4,0)="","—",VLOOKUP($A12,Accounts!$A$7:$D$566,4,0)),"—"))</f>
         <v>علی احمدی (نمونه)</v>
       </c>
-      <c r="C12" s="8" t="s">
-        <v>315</v>
-      </c>
-      <c r="D12" s="8" t="s">
-        <v>170</v>
-      </c>
-      <c r="E12" s="8" t="s">
-        <v>367</v>
-      </c>
+      <c r="C12" s="8"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="8"/>
       <c r="F12" s="8"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
@@ -19107,112 +19131,52 @@
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A7" s="13" t="s">
-        <v>428</v>
-      </c>
-      <c r="B7" s="7" t="s">
-        <v>133</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>142</v>
-      </c>
-      <c r="D7" s="7" t="s">
-        <v>1449</v>
-      </c>
-      <c r="E7" s="7" t="s">
-        <v>429</v>
-      </c>
-      <c r="F7" s="7" t="s">
-        <v>430</v>
-      </c>
-      <c r="G7" s="7" t="s">
-        <v>431</v>
-      </c>
-      <c r="H7" s="7" t="s">
-        <v>432</v>
-      </c>
+      <c r="A7" s="13"/>
+      <c r="B7" s="7"/>
+      <c r="C7" s="7"/>
+      <c r="D7" s="7"/>
+      <c r="E7" s="7"/>
+      <c r="F7" s="7"/>
+      <c r="G7" s="7"/>
+      <c r="H7" s="7"/>
       <c r="I7" s="13" t="str">
         <f t="shared" ref="I7:I70" si="0">IF($A7="","",IF(LEFT(UPPER(TRIM($A7)),2)="SL","فروشنده",IF(LEFT(UPPER(TRIM($A7)),3)="CAP","سرمایه و آورده صاحبان",IF(LEFT(UPPER(TRIM($A7)),1)="F","دارایی ثابت",IF(LEFT(UPPER(TRIM($A7)),1)="L","وام و تسهیلات",IF(LEFT(UPPER(TRIM($A7)),1)="C","مشتری",IF(LEFT(UPPER(TRIM($A7)),1)="S","تأمین‌کننده",IF(LEFT(UPPER(TRIM($A7)),1)="E","کارمند",IF(LEFT(UPPER(TRIM($A7)),1)="X","سایر حساب","")))))))))</f>
         <v>مشتری</v>
       </c>
-      <c r="J7" s="7" t="s">
-        <v>147</v>
-      </c>
-      <c r="K7" s="7" t="s">
-        <v>148</v>
-      </c>
+      <c r="J7" s="7"/>
+      <c r="K7" s="7"/>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A8" s="13" t="s">
-        <v>433</v>
-      </c>
-      <c r="B8" s="7" t="s">
-        <v>133</v>
-      </c>
-      <c r="C8" s="7" t="s">
-        <v>149</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>1450</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>434</v>
-      </c>
-      <c r="F8" s="7" t="s">
-        <v>435</v>
-      </c>
-      <c r="G8" s="7" t="s">
-        <v>436</v>
-      </c>
-      <c r="H8" s="7" t="s">
-        <v>437</v>
-      </c>
+      <c r="A8" s="13"/>
+      <c r="B8" s="7"/>
+      <c r="C8" s="7"/>
+      <c r="D8" s="7"/>
+      <c r="E8" s="7"/>
+      <c r="F8" s="7"/>
+      <c r="G8" s="7"/>
+      <c r="H8" s="7"/>
       <c r="I8" s="13" t="str">
         <f t="shared" si="0"/>
         <v>مشتری</v>
       </c>
-      <c r="J8" s="7" t="s">
-        <v>147</v>
-      </c>
-      <c r="K8" s="7" t="s">
-        <v>148</v>
-      </c>
+      <c r="J8" s="7"/>
+      <c r="K8" s="7"/>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A9" s="13" t="s">
-        <v>438</v>
-      </c>
-      <c r="B9" s="7" t="s">
-        <v>133</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>157</v>
-      </c>
-      <c r="D9" s="7" t="s">
-        <v>1451</v>
-      </c>
-      <c r="E9" s="7" t="s">
-        <v>439</v>
-      </c>
-      <c r="F9" s="7" t="s">
-        <v>440</v>
-      </c>
-      <c r="G9" s="7" t="s">
-        <v>441</v>
-      </c>
-      <c r="H9" s="7" t="s">
-        <v>437</v>
-      </c>
+      <c r="A9" s="13"/>
+      <c r="B9" s="7"/>
+      <c r="C9" s="7"/>
+      <c r="D9" s="7"/>
+      <c r="E9" s="7"/>
+      <c r="F9" s="7"/>
+      <c r="G9" s="7"/>
+      <c r="H9" s="7"/>
       <c r="I9" s="13" t="str">
         <f t="shared" si="0"/>
         <v>مشتری</v>
       </c>
-      <c r="J9" s="7" t="s">
-        <v>155</v>
-      </c>
-      <c r="K9" s="7" t="s">
-        <v>156</v>
-      </c>
+      <c r="J9" s="7"/>
+      <c r="K9" s="7"/>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A10" s="13" t="s">
@@ -23085,32 +23049,20 @@
       </c>
     </row>
     <row r="210" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A210" s="13" t="s">
-        <v>643</v>
-      </c>
-      <c r="B210" s="7" t="s">
-        <v>133</v>
-      </c>
+      <c r="A210" s="13"/>
+      <c r="B210" s="7"/>
       <c r="C210" s="7"/>
-      <c r="D210" s="7" t="s">
-        <v>1544</v>
-      </c>
+      <c r="D210" s="7"/>
       <c r="E210" s="7"/>
       <c r="F210" s="7"/>
       <c r="G210" s="7"/>
-      <c r="H210" s="7" t="s">
-        <v>437</v>
-      </c>
+      <c r="H210" s="7"/>
       <c r="I210" s="13" t="str">
         <f t="shared" si="3"/>
         <v>فروشنده</v>
       </c>
-      <c r="J210" s="7" t="s">
-        <v>162</v>
-      </c>
-      <c r="K210" s="7" t="s">
-        <v>156</v>
-      </c>
+      <c r="J210" s="7"/>
+      <c r="K210" s="7"/>
     </row>
     <row r="211" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A211" s="13" t="s">
@@ -26823,72 +26775,36 @@
       </c>
     </row>
     <row r="411" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A411" s="13" t="s">
-        <v>364</v>
-      </c>
-      <c r="B411" s="7" t="s">
-        <v>135</v>
-      </c>
-      <c r="C411" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="D411" s="7" t="s">
-        <v>855</v>
-      </c>
+      <c r="A411" s="13"/>
+      <c r="B411" s="7"/>
+      <c r="C411" s="7"/>
+      <c r="D411" s="7"/>
       <c r="E411" s="7"/>
-      <c r="F411" s="7" t="s">
-        <v>856</v>
-      </c>
-      <c r="G411" s="7" t="s">
-        <v>642</v>
-      </c>
-      <c r="H411" s="7" t="s">
-        <v>857</v>
-      </c>
+      <c r="F411" s="7"/>
+      <c r="G411" s="7"/>
+      <c r="H411" s="7"/>
       <c r="I411" s="13" t="str">
         <f t="shared" si="6"/>
         <v>کارمند</v>
       </c>
-      <c r="J411" s="7" t="s">
-        <v>155</v>
-      </c>
-      <c r="K411" s="7" t="s">
-        <v>163</v>
-      </c>
+      <c r="J411" s="7"/>
+      <c r="K411" s="7"/>
     </row>
     <row r="412" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A412" s="13" t="s">
-        <v>366</v>
-      </c>
-      <c r="B412" s="7" t="s">
-        <v>135</v>
-      </c>
-      <c r="C412" s="7" t="s">
-        <v>170</v>
-      </c>
-      <c r="D412" s="7" t="s">
-        <v>858</v>
-      </c>
+      <c r="A412" s="13"/>
+      <c r="B412" s="7"/>
+      <c r="C412" s="7"/>
+      <c r="D412" s="7"/>
       <c r="E412" s="7"/>
-      <c r="F412" s="7" t="s">
-        <v>859</v>
-      </c>
-      <c r="G412" s="7" t="s">
-        <v>642</v>
-      </c>
-      <c r="H412" s="7" t="s">
-        <v>857</v>
-      </c>
+      <c r="F412" s="7"/>
+      <c r="G412" s="7"/>
+      <c r="H412" s="7"/>
       <c r="I412" s="13" t="str">
         <f t="shared" si="6"/>
         <v>کارمند</v>
       </c>
-      <c r="J412" s="7" t="s">
-        <v>155</v>
-      </c>
-      <c r="K412" s="7" t="s">
-        <v>163</v>
-      </c>
+      <c r="J412" s="7"/>
+      <c r="K412" s="7"/>
     </row>
     <row r="413" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A413" s="13" t="s">
@@ -28599,96 +28515,52 @@
       <c r="K506" s="7"/>
     </row>
     <row r="507" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A507" s="13" t="s">
-        <v>910</v>
-      </c>
-      <c r="B507" s="7" t="s">
-        <v>137</v>
-      </c>
-      <c r="C507" s="7" t="s">
-        <v>144</v>
-      </c>
-      <c r="D507" s="7" t="s">
-        <v>911</v>
-      </c>
+      <c r="A507" s="13"/>
+      <c r="B507" s="7"/>
+      <c r="C507" s="7"/>
+      <c r="D507" s="7"/>
       <c r="E507" s="7"/>
       <c r="F507" s="7"/>
-      <c r="G507" s="7" t="s">
-        <v>743</v>
-      </c>
-      <c r="H507" s="7" t="s">
-        <v>912</v>
-      </c>
+      <c r="G507" s="7"/>
+      <c r="H507" s="7"/>
       <c r="I507" s="13" t="str">
         <f t="shared" si="7"/>
         <v>دارایی ثابت</v>
       </c>
-      <c r="J507" s="7" t="s">
-        <v>155</v>
-      </c>
-      <c r="K507" s="7" t="s">
-        <v>148</v>
-      </c>
+      <c r="J507" s="7"/>
+      <c r="K507" s="7"/>
     </row>
     <row r="508" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A508" s="13" t="s">
-        <v>913</v>
-      </c>
-      <c r="B508" s="7" t="s">
-        <v>137</v>
-      </c>
-      <c r="C508" s="7" t="s">
-        <v>152</v>
-      </c>
-      <c r="D508" s="7" t="s">
-        <v>914</v>
-      </c>
+      <c r="A508" s="13"/>
+      <c r="B508" s="7"/>
+      <c r="C508" s="7"/>
+      <c r="D508" s="7"/>
       <c r="E508" s="7"/>
       <c r="F508" s="7"/>
       <c r="G508" s="7"/>
-      <c r="H508" s="7" t="s">
-        <v>915</v>
-      </c>
+      <c r="H508" s="7"/>
       <c r="I508" s="13" t="str">
         <f t="shared" si="7"/>
         <v>دارایی ثابت</v>
       </c>
-      <c r="J508" s="7" t="s">
-        <v>155</v>
-      </c>
-      <c r="K508" s="7" t="s">
-        <v>156</v>
-      </c>
+      <c r="J508" s="7"/>
+      <c r="K508" s="7"/>
     </row>
     <row r="509" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A509" s="13" t="s">
-        <v>916</v>
-      </c>
-      <c r="B509" s="7" t="s">
-        <v>137</v>
-      </c>
-      <c r="C509" s="7" t="s">
-        <v>160</v>
-      </c>
-      <c r="D509" s="7" t="s">
-        <v>917</v>
-      </c>
+      <c r="A509" s="13"/>
+      <c r="B509" s="7"/>
+      <c r="C509" s="7"/>
+      <c r="D509" s="7"/>
       <c r="E509" s="7"/>
       <c r="F509" s="7"/>
       <c r="G509" s="7"/>
-      <c r="H509" s="7" t="s">
-        <v>915</v>
-      </c>
+      <c r="H509" s="7"/>
       <c r="I509" s="13" t="str">
         <f t="shared" si="7"/>
         <v>دارایی ثابت</v>
       </c>
-      <c r="J509" s="7" t="s">
-        <v>155</v>
-      </c>
-      <c r="K509" s="7" t="s">
-        <v>156</v>
-      </c>
+      <c r="J509" s="7"/>
+      <c r="K509" s="7"/>
     </row>
     <row r="510" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A510" s="13" t="s">
@@ -29177,34 +29049,20 @@
       <c r="K536" s="7"/>
     </row>
     <row r="537" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A537" s="13" t="s">
-        <v>945</v>
-      </c>
-      <c r="B537" s="7" t="s">
-        <v>138</v>
-      </c>
-      <c r="C537" s="7" t="s">
-        <v>145</v>
-      </c>
-      <c r="D537" s="7" t="s">
-        <v>946</v>
-      </c>
+      <c r="A537" s="13"/>
+      <c r="B537" s="7"/>
+      <c r="C537" s="7"/>
+      <c r="D537" s="7"/>
       <c r="E537" s="7"/>
       <c r="F537" s="7"/>
       <c r="G537" s="7"/>
-      <c r="H537" s="7" t="s">
-        <v>947</v>
-      </c>
+      <c r="H537" s="7"/>
       <c r="I537" s="13" t="str">
         <f t="shared" si="8"/>
         <v>وام و تسهیلات</v>
       </c>
-      <c r="J537" s="7" t="s">
-        <v>147</v>
-      </c>
-      <c r="K537" s="7" t="s">
-        <v>148</v>
-      </c>
+      <c r="J537" s="7"/>
+      <c r="K537" s="7"/>
     </row>
     <row r="538" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A538" s="13" t="s">
@@ -29549,34 +29407,20 @@
       <c r="K556" s="7"/>
     </row>
     <row r="557" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A557" s="13" t="s">
-        <v>967</v>
-      </c>
-      <c r="B557" s="7" t="s">
-        <v>139</v>
-      </c>
-      <c r="C557" s="7" t="s">
-        <v>146</v>
-      </c>
-      <c r="D557" s="7" t="s">
-        <v>968</v>
-      </c>
+      <c r="A557" s="13"/>
+      <c r="B557" s="7"/>
+      <c r="C557" s="7"/>
+      <c r="D557" s="7"/>
       <c r="E557" s="7"/>
       <c r="F557" s="7"/>
       <c r="G557" s="7"/>
-      <c r="H557" s="7" t="s">
-        <v>969</v>
-      </c>
+      <c r="H557" s="7"/>
       <c r="I557" s="13" t="str">
         <f t="shared" si="8"/>
         <v>سرمایه و آورده صاحبان</v>
       </c>
-      <c r="J557" s="7" t="s">
-        <v>147</v>
-      </c>
-      <c r="K557" s="7" t="s">
-        <v>148</v>
-      </c>
+      <c r="J557" s="7"/>
+      <c r="K557" s="7"/>
     </row>
     <row r="558" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A558" s="13" t="s">

</xml_diff>